<commit_message>
RUN-2026-01 G1b pass_with_conditions: comparator countries, LIM-0027, LIM-0028, E14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/RUN-2026-01/G1b_comparators.xlsx
+++ b/review/RUN-2026-01/G1b_comparators.xlsx
@@ -521,8 +521,16 @@
           <t>This sets what the policy options can draw on. Each issue deliberately includes a stalled or mixed case, so lessons are not drawn only from apparent successes.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0008</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -555,8 +563,16 @@
           <t>Without it, RI-FMW-001 has no case where removal has actually been applied, which is the most useful one for North Macedonia.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0008</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -589,8 +605,16 @@
           <t>Using it may give sharper evidence on Montenegro, but would put a restricted document in a public repository.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0008</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -623,8 +647,16 @@
           <t>Sets expectations: the pilot will show what was tried and what resulted, with limited proof of what caused it.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0008</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -657,8 +689,16 @@
           <t>Acquisition starts on these lines only.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>accept_recommendation</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Sofia, 30 Oct 2026, GATE-0008</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H6"/>

</xml_diff>